<commit_message>
Ultimate UI Redesign: Expanded Wheel Catalog (18 SKUs), High-Impact Typography, and Professional B2B Components
</commit_message>
<xml_diff>
--- a/Quotation_MOZA_CONSULTORIA_20260522.xlsx
+++ b/Quotation_MOZA_CONSULTORIA_20260522.xlsx
@@ -488,11 +488,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="43" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -682,40 +682,140 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9">
-        <f>SUM(A13:A16)</f>
-        <v/>
-      </c>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="10">
-        <f>SUM(C13:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="11">
-        <f>SUM(D13:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="9" t="n"/>
+      <c r="A17" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Customized Ceramic Mug (150ml)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="E17" s="5">
+        <f>C17*D17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Customized Ceramic Mug (Belly Model, 300ml)</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="E18" s="8">
+        <f>C18*D18</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Customized Ceramic Mug (250ml)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="E19" s="5">
+        <f>C19*D19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Glass Espresso Coffee Cup (130ml)</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>72</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="E20" s="8">
+        <f>C20*D20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Glass Espresso Coffee Cup (240ml)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="E21" s="5">
+        <f>C21*D21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9">
+        <f>SUM(A13:A21)</f>
+        <v/>
+      </c>
+      <c r="B22" s="9" t="n"/>
+      <c r="C22" s="10">
+        <f>SUM(C13:C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="11">
+        <f>SUM(D13:D21)</f>
+        <v/>
+      </c>
+      <c r="E22" s="9" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Trade Terms:</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Validity:</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>30 Days</t>
         </is>

</xml_diff>